<commit_message>
Updated code and files for Sprint 3, now with backend for Study Space seat tracking
</commit_message>
<xml_diff>
--- a/src/data/resteraunt_reviews.xlsx
+++ b/src/data/resteraunt_reviews.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\CP317\Group Assignment\HawkMaps\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C484D11-C8A6-40EC-9509-9E254A005C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A033D54-BB67-41A8-9E04-BF83E071CB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Condensed Campus Map" sheetId="1" r:id="rId1"/>
@@ -23,15 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="27">
   <si>
     <t>Campus Locations &amp; Coordinates (Condensed Format)</t>
   </si>
   <si>
     <t>Building</t>
-  </si>
-  <si>
-    <t>Dining Hall</t>
   </si>
   <si>
     <t>Byte 75 Coffee &amp; Social</t>
@@ -214,9 +211,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -231,6 +225,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,700 +535,652 @@
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="3" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="9" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="6">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="7">
-        <v>5</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="6">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="6" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="7">
-        <v>3</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="C6" s="6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="3" t="s">
+    <row r="7" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="7">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="7">
-        <v>5</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C8" s="6">
+        <v>3</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E8" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="s">
+    <row r="9" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="7">
-        <v>3</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="6">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="3" t="s">
+    <row r="10" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="6">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="7">
-        <v>5</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="6">
+        <v>3</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E11" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="7">
-        <v>3</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C12" s="6">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="3" t="s">
+    <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="6">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="7">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="3" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="7">
-        <v>5</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C14" s="6">
+        <v>3</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E14" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="3" t="s">
+    <row r="15" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="7">
-        <v>3</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="3" t="s">
+    <row r="16" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6">
+        <v>5</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="7">
-        <v>1</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="7">
-        <v>5</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="C17" s="6">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E17" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="18" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="7">
-        <v>3</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="3" t="s">
+    <row r="19" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="6">
+        <v>5</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="7">
-        <v>1</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E19" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="7">
-        <v>5</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="C20" s="6">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="21" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="7">
-        <v>3</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E21" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B21" s="3" t="s">
+    <row r="22" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="6">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="7">
-        <v>1</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="E22" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    </row>
+    <row r="23" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="7">
-        <v>5</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="C23" s="6">
+        <v>3</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E23" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="24" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="7">
-        <v>3</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E24" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" s="3" t="s">
+    <row r="25" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="6">
+        <v>5</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="7">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="E25" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E24" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+    </row>
+    <row r="26" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="7">
-        <v>5</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="C26" s="6">
+        <v>3</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+    <row r="27" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="7">
-        <v>3</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="C27" s="6">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E27" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="3" t="s">
+    <row r="28" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="6">
+        <v>5</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="7">
-        <v>1</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="E28" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+    </row>
+    <row r="29" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B29" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="7">
-        <v>5</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="C29" s="6">
+        <v>3</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E29" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+    <row r="30" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B30" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C29" s="7">
-        <v>3</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="C30" s="6">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E30" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B30" s="3" t="s">
+    <row r="31" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="6">
+        <v>5</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C30" s="7">
-        <v>1</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="E31" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+    </row>
+    <row r="32" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B32" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="7">
-        <v>5</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="C32" s="6">
+        <v>3</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+    <row r="33" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B33" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="7">
-        <v>3</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="C33" s="6">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E33" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" s="3" t="s">
+    <row r="34" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="6">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="7">
-        <v>1</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="E34" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+    </row>
+    <row r="35" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="7">
-        <v>5</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="C35" s="6">
+        <v>3</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E35" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="36" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B36" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="7">
-        <v>3</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="C36" s="6">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E36" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" s="3" t="s">
+    <row r="37" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="6">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="7">
-        <v>1</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="E37" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E36" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+    </row>
+    <row r="38" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="7">
-        <v>5</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="C38" s="6">
+        <v>3</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E38" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+    <row r="39" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="7">
-        <v>3</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="C39" s="6">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E39" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="7">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C40" s="7">
-        <v>5</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C41" s="7">
-        <v>3</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="7">
-        <v>1</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
+    <row r="40" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A3:E3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="1">

</xml_diff>